<commit_message>
auto: Daily attendance & approvals update 9AM
</commit_message>
<xml_diff>
--- a/Padron_Trabajadores_GZG.xlsx
+++ b/Padron_Trabajadores_GZG.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GZG Minerales 2026\Desktop\GZG\Sistema_Asistencia_GZG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D3649AD-6EF1-4394-8C7C-57C3F3F91EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FBABBEB-F31D-457D-92ED-16E3561BBE7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="210">
   <si>
     <t>PADRÓN OFICIAL DE TRABAJADORES Y PERSONAL REGISTRADO - GZG MINERALES</t>
   </si>
@@ -645,6 +645,15 @@
   </si>
   <si>
     <t>73577356</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOLORZANO AVILA </t>
+  </si>
+  <si>
+    <t>MANUEL SEBASTIAN</t>
+  </si>
+  <si>
+    <t>71620681</t>
   </si>
 </sst>
 </file>
@@ -1084,8 +1093,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1151,7 +1159,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -1177,7 +1185,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -1203,7 +1211,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -1229,7 +1237,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -1255,7 +1263,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
@@ -1281,7 +1289,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>30</v>
       </c>
@@ -1307,7 +1315,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>33</v>
       </c>
@@ -1333,7 +1341,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>37</v>
       </c>
@@ -1359,7 +1367,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>40</v>
       </c>
@@ -1385,7 +1393,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>43</v>
       </c>
@@ -1411,7 +1419,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>46</v>
       </c>
@@ -1437,7 +1445,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>49</v>
       </c>
@@ -1463,7 +1471,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>52</v>
       </c>
@@ -1489,7 +1497,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>55</v>
       </c>
@@ -1515,7 +1523,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>58</v>
       </c>
@@ -1541,7 +1549,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>62</v>
       </c>
@@ -1567,7 +1575,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>66</v>
       </c>
@@ -1593,7 +1601,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>69</v>
       </c>
@@ -1619,7 +1627,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>72</v>
       </c>
@@ -1645,7 +1653,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>75</v>
       </c>
@@ -1671,7 +1679,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>78</v>
       </c>
@@ -1697,7 +1705,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>81</v>
       </c>
@@ -1723,7 +1731,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>83</v>
       </c>
@@ -1749,7 +1757,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>86</v>
       </c>
@@ -1775,7 +1783,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>89</v>
       </c>
@@ -1801,7 +1809,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>94</v>
       </c>
@@ -1827,7 +1835,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>97</v>
       </c>
@@ -1853,7 +1861,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>100</v>
       </c>
@@ -1879,7 +1887,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>104</v>
       </c>
@@ -1905,7 +1913,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>107</v>
       </c>
@@ -1931,7 +1939,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>110</v>
       </c>
@@ -1957,7 +1965,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>113</v>
       </c>
@@ -1983,7 +1991,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>116</v>
       </c>
@@ -2009,7 +2017,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>118</v>
       </c>
@@ -2035,7 +2043,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>122</v>
       </c>
@@ -2061,7 +2069,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>126</v>
       </c>
@@ -2087,7 +2095,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>129</v>
       </c>
@@ -2113,7 +2121,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>132</v>
       </c>
@@ -2139,7 +2147,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>135</v>
       </c>
@@ -2165,7 +2173,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>138</v>
       </c>
@@ -2191,7 +2199,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>141</v>
       </c>
@@ -2217,7 +2225,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>144</v>
       </c>
@@ -2243,7 +2251,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>147</v>
       </c>
@@ -2269,7 +2277,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>151</v>
       </c>
@@ -2295,7 +2303,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>154</v>
       </c>
@@ -2321,7 +2329,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>157</v>
       </c>
@@ -2347,7 +2355,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>161</v>
       </c>
@@ -2373,7 +2381,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>164</v>
       </c>
@@ -2399,7 +2407,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>167</v>
       </c>
@@ -2425,7 +2433,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>170</v>
       </c>
@@ -2451,7 +2459,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>173</v>
       </c>
@@ -2477,7 +2485,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>176</v>
       </c>
@@ -2503,7 +2511,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>179</v>
       </c>
@@ -2529,7 +2537,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>182</v>
       </c>
@@ -2581,14 +2589,34 @@
         <v>195</v>
       </c>
     </row>
+    <row r="59" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:H58" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="TEJADA VASQUEZ"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A3:H58" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>

</xml_diff>